<commit_message>
fix(ci): Upgrade GitHub Actions to Node 22 to fix deprecation warning and add generateFinalReport method to load-test ExcelReporter
</commit_message>
<xml_diff>
--- a/load-test/excel/Load_Testing_Report.xlsx
+++ b/load-test/excel/Load_Testing_Report.xlsx
@@ -25,7 +25,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-08-06T05:36:04.298Z</t>
+    <t>2026-08-06T05:43:54.498Z</t>
   </si>
   <si>
     <t>Target System URL</t>
@@ -52,7 +52,7 @@
     <t>Requests Per Second (RPS)</t>
   </si>
   <si>
-    <t>2419.31 req/sec</t>
+    <t>1901.62 req/sec</t>
   </si>
   <si>
     <t>Minimum Response Time</t>
@@ -64,19 +64,19 @@
     <t>Average Response Time</t>
   </si>
   <si>
-    <t>41.05 ms</t>
+    <t>52.26 ms</t>
   </si>
   <si>
     <t>Maximum Response Time</t>
   </si>
   <si>
-    <t>2784 ms</t>
+    <t>1028 ms</t>
   </si>
   <si>
     <t>50th Percentile Latency (p50)</t>
   </si>
   <si>
-    <t>23 ms</t>
+    <t>32 ms</t>
   </si>
   <si>
     <t>95th Percentile Latency (p95)</t>
@@ -88,7 +88,7 @@
     <t>99th Percentile Latency (p99)</t>
   </si>
   <si>
-    <t>421 ms</t>
+    <t>377 ms</t>
   </si>
   <si>
     <t>Success 2xx Responses</t>
@@ -121,7 +121,7 @@
     <t>Minimum (Fastest)</t>
   </si>
   <si>
-    <t>2419.31 req/s</t>
+    <t>1901.62 req/s</t>
   </si>
   <si>
     <t>Average (Mean)</t>
@@ -133,7 +133,7 @@
     <t>90th Percentile (p90)</t>
   </si>
   <si>
-    <t>62 ms</t>
+    <t>103 ms</t>
   </si>
   <si>
     <t>95th Percentile (p95)</t>
@@ -196,7 +196,7 @@
     <t>Details</t>
   </si>
   <si>
-    <t>2026-08-06T05:36:04.305Z</t>
+    <t>2026-08-06T05:43:54.503Z</t>
   </si>
   <si>
     <t>Ramp-up (100 VUs)</t>
@@ -211,13 +211,13 @@
     <t>Sustained Load (60s)</t>
   </si>
   <si>
-    <t>Executed continuous requests at 2419.31 RPS</t>
+    <t>Executed continuous requests at 1901.62 RPS</t>
   </si>
   <si>
     <t>Metrics Aggregation</t>
   </si>
   <si>
-    <t>Min: 6ms, Avg: 41.05ms, Max: 2784ms</t>
+    <t>Min: 6ms, Avg: 52.26ms, Max: 1028ms</t>
   </si>
 </sst>
 </file>
@@ -677,7 +677,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>145142</v>
+        <v>114083</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -741,7 +741,7 @@
         <v>25</v>
       </c>
       <c r="B14">
-        <v>145142</v>
+        <v>114083</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -911,7 +911,7 @@
         <v>49</v>
       </c>
       <c r="C2">
-        <v>24190</v>
+        <v>19013</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
@@ -928,7 +928,7 @@
         <v>49</v>
       </c>
       <c r="C3">
-        <v>24190</v>
+        <v>19013</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
@@ -945,7 +945,7 @@
         <v>49</v>
       </c>
       <c r="C4">
-        <v>24190</v>
+        <v>19013</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
@@ -962,7 +962,7 @@
         <v>49</v>
       </c>
       <c r="C5">
-        <v>24190</v>
+        <v>19013</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -979,7 +979,7 @@
         <v>49</v>
       </c>
       <c r="C6">
-        <v>24190</v>
+        <v>19013</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
@@ -996,7 +996,7 @@
         <v>49</v>
       </c>
       <c r="C7">
-        <v>24190</v>
+        <v>19013</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>

</xml_diff>